<commit_message>
Add Docker full-stack packaging for Dad Windows laptop hosting.
Ship postgres+api+ui Compose, Research/Final Master mounts, Windows setup and US update docs, and PowerShell start/update helpers so the app runs with Docker Desktop only.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/portfolio_snapshots/Portfolio_2025.xlsx
+++ b/data/raw/portfolio_snapshots/Portfolio_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c3b54154a9f56a2/Samir/Research/Portfolio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c3b54154a9f56a2/Samir/Research/Portfolio/Portfolio Yearly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1606" documentId="8_{EDF33660-9B23-4888-B529-2B640994E33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9DC65ED-E92E-43CC-8698-0BC376095E5A}"/>
+  <xr:revisionPtr revIDLastSave="1611" documentId="8_{EDF33660-9B23-4888-B529-2B640994E33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F61FA10-3BF9-4920-9B74-72AED1D5B5F6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="16" activeTab="23" xr2:uid="{D1491BFC-AA9E-4856-B603-CFD392162666}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="6" xr2:uid="{D1491BFC-AA9E-4856-B603-CFD392162666}"/>
   </bookViews>
   <sheets>
     <sheet name="01Jan25" sheetId="51" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="101">
   <si>
     <t>Model Portfolio</t>
   </si>
@@ -180,9 +180,6 @@
   </si>
   <si>
     <t>Rates of 24-03-2025</t>
-  </si>
-  <si>
-    <t>Buy 1952@107.67</t>
   </si>
   <si>
     <t>Sell 405@519.03 = 210207</t>
@@ -361,6 +358,12 @@
   <si>
     <t>Sell 1247</t>
   </si>
+  <si>
+    <t>Sell 2568@179.7 = 461469</t>
+  </si>
+  <si>
+    <t>Buy 4295+1952@107.67</t>
+  </si>
 </sst>
 </file>
 
@@ -420,10 +423,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1239,7 +1238,7 @@
         <v>45782</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -1345,7 +1344,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" s="4">
         <v>724</v>
@@ -1363,7 +1362,7 @@
       </c>
       <c r="F8"/>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H8"/>
       <c r="I8"/>
@@ -1556,7 +1555,7 @@
       </c>
       <c r="F16"/>
       <c r="G16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H16"/>
       <c r="I16"/>
@@ -1678,7 +1677,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -1739,7 +1738,7 @@
         <v>45797</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -1816,7 +1815,7 @@
       </c>
       <c r="F6"/>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -1847,7 +1846,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -1871,7 +1870,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289</f>
@@ -1890,7 +1889,7 @@
       </c>
       <c r="F9"/>
       <c r="G9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
@@ -2059,7 +2058,7 @@
       </c>
       <c r="F16"/>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H16"/>
       <c r="I16"/>
@@ -2181,7 +2180,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -2243,7 +2242,7 @@
         <v>45810</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -2320,7 +2319,7 @@
       </c>
       <c r="F6"/>
       <c r="G6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -2351,7 +2350,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -2375,7 +2374,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144</f>
@@ -2394,7 +2393,7 @@
       </c>
       <c r="F9"/>
       <c r="G9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
@@ -2683,7 +2682,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -2745,7 +2744,7 @@
         <v>45810</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -2851,7 +2850,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -2875,7 +2874,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144</f>
@@ -2966,7 +2965,7 @@
       </c>
       <c r="F12"/>
       <c r="G12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H12"/>
       <c r="I12"/>
@@ -3184,7 +3183,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -3246,7 +3245,7 @@
         <v>45810</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -3352,7 +3351,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -3376,7 +3375,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144</f>
@@ -3745,7 +3744,7 @@
         <v>45887</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -3822,7 +3821,7 @@
       </c>
       <c r="F6"/>
       <c r="G6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -3853,7 +3852,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -3877,7 +3876,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144</f>
@@ -3968,7 +3967,7 @@
       </c>
       <c r="F12"/>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H12"/>
       <c r="I12"/>
@@ -4186,7 +4185,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -4248,7 +4247,7 @@
         <v>45904</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -4325,7 +4324,7 @@
       </c>
       <c r="F6"/>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -4356,7 +4355,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -4380,7 +4379,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144</f>
@@ -4687,7 +4686,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -4749,7 +4748,7 @@
         <v>45909</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -4855,7 +4854,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -4879,7 +4878,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144</f>
@@ -4970,7 +4969,7 @@
       </c>
       <c r="F12"/>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H12"/>
       <c r="I12"/>
@@ -5188,7 +5187,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -5250,7 +5249,7 @@
         <v>45957</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -5356,7 +5355,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -5380,7 +5379,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144+275</f>
@@ -5399,7 +5398,7 @@
       </c>
       <c r="F9"/>
       <c r="G9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
@@ -5689,7 +5688,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -5751,7 +5750,7 @@
         <v>45959</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -5857,7 +5856,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -5881,7 +5880,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144+275</f>
@@ -5905,7 +5904,7 @@
     </row>
     <row r="10" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B10" s="4">
         <v>3770</v>
@@ -5923,7 +5922,7 @@
       </c>
       <c r="F10"/>
       <c r="G10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H10"/>
       <c r="I10"/>
@@ -6213,7 +6212,7 @@
       </c>
       <c r="F22"/>
       <c r="G22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H22"/>
       <c r="I22"/>
@@ -6768,7 +6767,7 @@
         <v>45968</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -6845,7 +6844,7 @@
       </c>
       <c r="F6"/>
       <c r="G6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -6876,7 +6875,7 @@
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -6900,7 +6899,7 @@
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144+275</f>
@@ -6924,7 +6923,7 @@
     </row>
     <row r="10" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B10" s="4">
         <v>3770</v>
@@ -7014,7 +7013,7 @@
       </c>
       <c r="F13"/>
       <c r="G13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H13"/>
       <c r="I13"/>
@@ -7112,7 +7111,7 @@
       </c>
       <c r="F17"/>
       <c r="G17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H17"/>
       <c r="I17"/>
@@ -7234,7 +7233,7 @@
       </c>
       <c r="F22"/>
       <c r="G22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H22"/>
       <c r="I22"/>
@@ -7296,7 +7295,7 @@
         <v>45978</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -7402,7 +7401,7 @@
     </row>
     <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4">
         <f>130+126+33+57+173+130</f>
@@ -7426,7 +7425,7 @@
     </row>
     <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4">
         <f>724+289+144+275-367</f>
@@ -7445,14 +7444,14 @@
       </c>
       <c r="F9"/>
       <c r="G9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
     </row>
     <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B10" s="4">
         <v>3770</v>
@@ -7566,7 +7565,7 @@
       </c>
       <c r="F14"/>
       <c r="G14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H14"/>
       <c r="I14"/>
@@ -7713,7 +7712,7 @@
       </c>
       <c r="F20"/>
       <c r="G20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H20"/>
       <c r="I20"/>
@@ -7775,7 +7774,7 @@
         <v>45981</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -7809,7 +7808,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5" s="4">
         <v>2265</v>
@@ -7826,7 +7825,7 @@
         <v>3.0004655104092021E-2</v>
       </c>
       <c r="G5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -7903,7 +7902,7 @@
     </row>
     <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B9" s="4">
         <f>130+126+33+57+173+130</f>
@@ -7927,7 +7926,7 @@
     </row>
     <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" s="4">
         <f>724+289+144+275-367</f>
@@ -7951,7 +7950,7 @@
     </row>
     <row r="11" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" s="4">
         <v>3770</v>
@@ -8210,7 +8209,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -8272,7 +8271,7 @@
         <v>45999</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -8306,7 +8305,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5" s="4">
         <f>2265+463</f>
@@ -8324,7 +8323,7 @@
         <v>3.6121754021006126E-2</v>
       </c>
       <c r="G5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -8401,7 +8400,7 @@
     </row>
     <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B9" s="4">
         <f>130+126+33+57+173+130</f>
@@ -8425,7 +8424,7 @@
     </row>
     <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" s="4">
         <f>724+289+144+275-367</f>
@@ -8449,7 +8448,7 @@
     </row>
     <row r="11" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" s="4">
         <v>3770</v>
@@ -8708,7 +8707,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -8770,7 +8769,7 @@
         <v>46020</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -8804,7 +8803,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5" s="4">
         <f>2265+463</f>
@@ -8896,7 +8895,7 @@
     </row>
     <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B9" s="4">
         <f>130+126+33+57+173+130</f>
@@ -8920,7 +8919,7 @@
     </row>
     <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" s="4">
         <f>724+289+144+275-367</f>
@@ -8944,7 +8943,7 @@
     </row>
     <row r="11" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" s="4">
         <f>3770+209</f>
@@ -8963,7 +8962,7 @@
       </c>
       <c r="F11"/>
       <c r="G11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H11"/>
       <c r="I11"/>
@@ -9206,7 +9205,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -11447,7 +11446,9 @@
         <v>2.7418009176148703E-2</v>
       </c>
       <c r="F10"/>
-      <c r="G10"/>
+      <c r="G10" t="s">
+        <v>99</v>
+      </c>
       <c r="H10"/>
       <c r="I10"/>
     </row>
@@ -11663,7 +11664,7 @@
       </c>
       <c r="F19"/>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H19"/>
       <c r="I19" s="3"/>
@@ -11713,7 +11714,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -11851,7 +11852,7 @@
       </c>
       <c r="F6"/>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -12212,7 +12213,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -12273,7 +12274,7 @@
         <v>45776</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -12565,7 +12566,7 @@
       </c>
       <c r="F15"/>
       <c r="G15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H15"/>
       <c r="I15"/>
@@ -12711,7 +12712,7 @@
       </c>
       <c r="F21"/>
       <c r="G21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>

</xml_diff>